<commit_message>
Update: Mumbai-April-2026 by admin
</commit_message>
<xml_diff>
--- a/Mumbai-April-2026.xlsx
+++ b/Mumbai-April-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa30afadbe7955a4/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{3E5A074B-5161-4EB8-B06F-3025AB0F1620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C573E5A-BB11-4FCD-B4BB-1D9BC13424EA}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{3E5A074B-5161-4EB8-B06F-3025AB0F1620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{310E912A-11C8-4DF5-936C-36AAAF3366A9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="145">
   <si>
     <t>Model</t>
   </si>
@@ -466,9 +466,6 @@
   </si>
   <si>
     <t>MERCEDES E</t>
-  </si>
-  <si>
-    <t>XUV 401</t>
   </si>
   <si>
     <t>April</t>
@@ -789,6 +786,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1202,7 +1203,7 @@
         <v>88</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D2" s="11">
         <v>2026</v>
@@ -1286,7 +1287,7 @@
         <v>88</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D3" s="11">
         <v>2026</v>
@@ -1370,7 +1371,7 @@
         <v>88</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D4" s="11">
         <v>2026</v>
@@ -1454,7 +1455,7 @@
         <v>88</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" s="11">
         <v>2026</v>
@@ -1536,7 +1537,7 @@
         <v>88</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="11">
         <v>2026</v>
@@ -1618,7 +1619,7 @@
         <v>88</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D7" s="11">
         <v>2026</v>
@@ -1701,7 +1702,7 @@
         <v>88</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D8" s="11">
         <v>2026</v>
@@ -1785,7 +1786,7 @@
         <v>88</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D9" s="11">
         <v>2026</v>
@@ -1869,7 +1870,7 @@
         <v>88</v>
       </c>
       <c r="C10" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D10" s="11">
         <v>2026</v>
@@ -1952,7 +1953,7 @@
         <v>88</v>
       </c>
       <c r="C11" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D11" s="11">
         <v>2026</v>
@@ -2035,7 +2036,7 @@
         <v>88</v>
       </c>
       <c r="C12" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D12" s="11">
         <v>2026</v>
@@ -2118,7 +2119,7 @@
         <v>88</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D13" s="11">
         <v>2026</v>
@@ -2201,7 +2202,7 @@
         <v>88</v>
       </c>
       <c r="C14" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D14" s="11">
         <v>2026</v>
@@ -2282,7 +2283,7 @@
         <v>88</v>
       </c>
       <c r="C15" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D15" s="11">
         <v>2026</v>
@@ -2365,7 +2366,7 @@
         <v>88</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D16" s="11">
         <v>2026</v>
@@ -2448,7 +2449,7 @@
         <v>88</v>
       </c>
       <c r="C17" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D17" s="11">
         <v>2026</v>
@@ -2531,7 +2532,7 @@
         <v>88</v>
       </c>
       <c r="C18" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D18" s="11">
         <v>2026</v>
@@ -2614,7 +2615,7 @@
         <v>88</v>
       </c>
       <c r="C19" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D19" s="11">
         <v>2026</v>
@@ -2697,7 +2698,7 @@
         <v>88</v>
       </c>
       <c r="C20" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D20" s="11">
         <v>2026</v>
@@ -2780,7 +2781,7 @@
         <v>88</v>
       </c>
       <c r="C21" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D21" s="11">
         <v>2026</v>
@@ -2863,7 +2864,7 @@
         <v>88</v>
       </c>
       <c r="C22" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D22" s="11">
         <v>2026</v>
@@ -2946,7 +2947,7 @@
         <v>88</v>
       </c>
       <c r="C23" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D23" s="11">
         <v>2026</v>
@@ -3029,7 +3030,7 @@
         <v>88</v>
       </c>
       <c r="C24" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D24" s="11">
         <v>2026</v>
@@ -3112,7 +3113,7 @@
         <v>88</v>
       </c>
       <c r="C25" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D25" s="11">
         <v>2026</v>
@@ -3195,7 +3196,7 @@
         <v>88</v>
       </c>
       <c r="C26" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D26" s="11">
         <v>2026</v>
@@ -3278,7 +3279,7 @@
         <v>88</v>
       </c>
       <c r="C27" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D27" s="11">
         <v>2026</v>
@@ -3361,7 +3362,7 @@
         <v>88</v>
       </c>
       <c r="C28" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D28" s="11">
         <v>2026</v>
@@ -3446,7 +3447,7 @@
         <v>88</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D29" s="11">
         <v>2026</v>
@@ -3529,7 +3530,7 @@
         <v>88</v>
       </c>
       <c r="C30" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D30" s="11">
         <v>2026</v>
@@ -3612,7 +3613,7 @@
         <v>88</v>
       </c>
       <c r="C31" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D31" s="11">
         <v>2026</v>
@@ -3695,7 +3696,7 @@
         <v>88</v>
       </c>
       <c r="C32" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D32" s="11">
         <v>2026</v>
@@ -3778,7 +3779,7 @@
         <v>88</v>
       </c>
       <c r="C33" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D33" s="11">
         <v>2026</v>
@@ -3861,7 +3862,7 @@
         <v>88</v>
       </c>
       <c r="C34" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D34" s="11">
         <v>2026</v>
@@ -3944,7 +3945,7 @@
         <v>88</v>
       </c>
       <c r="C35" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D35" s="11">
         <v>2026</v>
@@ -4027,7 +4028,7 @@
         <v>88</v>
       </c>
       <c r="C36" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D36" s="11">
         <v>2026</v>
@@ -4110,7 +4111,7 @@
         <v>88</v>
       </c>
       <c r="C37" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D37" s="11">
         <v>2026</v>
@@ -4193,7 +4194,7 @@
         <v>88</v>
       </c>
       <c r="C38" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D38" s="11">
         <v>2026</v>
@@ -4276,7 +4277,7 @@
         <v>88</v>
       </c>
       <c r="C39" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D39" s="11">
         <v>2026</v>
@@ -4359,7 +4360,7 @@
         <v>88</v>
       </c>
       <c r="C40" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D40" s="11">
         <v>2026</v>
@@ -4440,7 +4441,7 @@
         <v>88</v>
       </c>
       <c r="C41" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D41" s="11">
         <v>2026</v>
@@ -4521,7 +4522,7 @@
         <v>88</v>
       </c>
       <c r="C42" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D42" s="11">
         <v>2026</v>
@@ -4602,7 +4603,7 @@
         <v>88</v>
       </c>
       <c r="C43" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D43" s="11">
         <v>2026</v>
@@ -4684,7 +4685,7 @@
         <v>88</v>
       </c>
       <c r="C44" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D44" s="11">
         <v>2026</v>
@@ -4765,7 +4766,7 @@
         <v>88</v>
       </c>
       <c r="C45" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D45" s="11">
         <v>2026</v>
@@ -4846,7 +4847,7 @@
         <v>88</v>
       </c>
       <c r="C46" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D46" s="11">
         <v>2026</v>
@@ -4927,7 +4928,7 @@
         <v>88</v>
       </c>
       <c r="C47" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D47" s="11">
         <v>2026</v>
@@ -5008,7 +5009,7 @@
         <v>88</v>
       </c>
       <c r="C48" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D48" s="11">
         <v>2026</v>
@@ -5089,7 +5090,7 @@
         <v>88</v>
       </c>
       <c r="C49" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D49" s="11">
         <v>2026</v>
@@ -5170,7 +5171,7 @@
         <v>88</v>
       </c>
       <c r="C50" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D50" s="11">
         <v>2026</v>
@@ -5251,7 +5252,7 @@
         <v>88</v>
       </c>
       <c r="C51" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D51" s="11">
         <v>2026</v>
@@ -5332,7 +5333,7 @@
         <v>88</v>
       </c>
       <c r="C52" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D52" s="11">
         <v>2026</v>
@@ -5413,7 +5414,7 @@
         <v>88</v>
       </c>
       <c r="C53" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D53" s="11">
         <v>2026</v>
@@ -5494,7 +5495,7 @@
         <v>88</v>
       </c>
       <c r="C54" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D54" s="11">
         <v>2026</v>
@@ -5577,7 +5578,7 @@
         <v>88</v>
       </c>
       <c r="C55" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D55" s="11">
         <v>2026</v>
@@ -5658,7 +5659,7 @@
         <v>88</v>
       </c>
       <c r="C56" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D56" s="11">
         <v>2026</v>
@@ -5739,7 +5740,7 @@
         <v>88</v>
       </c>
       <c r="C57" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D57" s="11">
         <v>2026</v>
@@ -5820,7 +5821,7 @@
         <v>88</v>
       </c>
       <c r="C58" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D58" s="11">
         <v>2026</v>
@@ -5901,7 +5902,7 @@
         <v>88</v>
       </c>
       <c r="C59" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D59" s="11">
         <v>2026</v>
@@ -5982,7 +5983,7 @@
         <v>88</v>
       </c>
       <c r="C60" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D60" s="11">
         <v>2026</v>
@@ -6063,7 +6064,7 @@
         <v>88</v>
       </c>
       <c r="C61" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D61" s="11">
         <v>2026</v>
@@ -6144,7 +6145,7 @@
         <v>88</v>
       </c>
       <c r="C62" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D62" s="11">
         <v>2026</v>
@@ -6226,7 +6227,7 @@
         <v>88</v>
       </c>
       <c r="C63" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D63" s="11">
         <v>2026</v>
@@ -6308,7 +6309,7 @@
         <v>88</v>
       </c>
       <c r="C64" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D64" s="11">
         <v>2026</v>
@@ -6390,7 +6391,7 @@
         <v>88</v>
       </c>
       <c r="C65" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D65" s="11">
         <v>2026</v>
@@ -6472,7 +6473,7 @@
         <v>88</v>
       </c>
       <c r="C66" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D66" s="11">
         <v>2026</v>
@@ -6554,7 +6555,7 @@
         <v>88</v>
       </c>
       <c r="C67" s="47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D67" s="11">
         <v>2026</v>
@@ -6563,7 +6564,7 @@
         <v>60</v>
       </c>
       <c r="F67" s="12" t="s">
-        <v>144</v>
+        <v>61</v>
       </c>
       <c r="G67" s="41" t="s">
         <v>122</v>

</xml_diff>